<commit_message>
Actualizar materias reales del 9o semestre con sus porcentajes de evaluacion
Co-authored-by: saospinap-bit <294225962+saospinap-bit@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mi-Sistema-de-Vida.xlsx
+++ b/Mi-Sistema-de-Vida.xlsx
@@ -6695,7 +6695,7 @@
     <row r="4">
       <c r="A4" s="42" t="inlineStr">
         <is>
-          <t>Diseno Estructural (PROYECTO)</t>
+          <t>Diseno Estructural</t>
         </is>
       </c>
       <c r="B4" s="20" t="n">
@@ -6725,7 +6725,7 @@
     <row r="5">
       <c r="A5" s="42" t="inlineStr">
         <is>
-          <t>Materia obligatoria 1</t>
+          <t>Uitoto</t>
         </is>
       </c>
       <c r="B5" s="20" t="n">
@@ -6755,7 +6755,7 @@
     <row r="6">
       <c r="A6" s="42" t="inlineStr">
         <is>
-          <t>Materia obligatoria 2</t>
+          <t>PEPI</t>
         </is>
       </c>
       <c r="B6" s="20" t="n">
@@ -6785,7 +6785,7 @@
     <row r="7">
       <c r="A7" s="42" t="inlineStr">
         <is>
-          <t>Materia obligatoria 3</t>
+          <t>Saneamiento Ambiental</t>
         </is>
       </c>
       <c r="B7" s="20" t="n">
@@ -6815,11 +6815,11 @@
     <row r="8">
       <c r="A8" s="42" t="inlineStr">
         <is>
-          <t>Materia optativa 1</t>
+          <t>Alcantarillados</t>
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="20">
         <f>'Calculadora Notas'!D78</f>
@@ -6845,11 +6845,11 @@
     <row r="9">
       <c r="A9" s="42" t="inlineStr">
         <is>
-          <t>Materia optativa 2</t>
+          <t>Fundamentos de Construccion</t>
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="20">
         <f>'Calculadora Notas'!D94</f>
@@ -6943,7 +6943,7 @@
     <row r="3">
       <c r="A3" s="47" t="inlineStr">
         <is>
-          <t>MATERIA: Diseno Estructural (PROYECTO)</t>
+          <t>MATERIA: Diseno Estructural</t>
         </is>
       </c>
     </row>
@@ -6972,10 +6972,12 @@
     <row r="5">
       <c r="A5" s="42" t="inlineStr">
         <is>
-          <t>Eval 1</t>
-        </is>
-      </c>
-      <c r="B5" s="49" t="n"/>
+          <t>Parcial 1</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C5" s="49" t="n"/>
       <c r="D5" s="20">
         <f>IFERROR(B5*C5/100,0)</f>
@@ -6985,10 +6987,12 @@
     <row r="6">
       <c r="A6" s="42" t="inlineStr">
         <is>
-          <t>Eval 2</t>
-        </is>
-      </c>
-      <c r="B6" s="49" t="n"/>
+          <t>Parcial 2</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C6" s="49" t="n"/>
       <c r="D6" s="20">
         <f>IFERROR(B6*C6/100,0)</f>
@@ -6998,10 +7002,12 @@
     <row r="7">
       <c r="A7" s="42" t="inlineStr">
         <is>
-          <t>Eval 3</t>
-        </is>
-      </c>
-      <c r="B7" s="49" t="n"/>
+          <t>Parcial 3</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C7" s="49" t="n"/>
       <c r="D7" s="20">
         <f>IFERROR(B7*C7/100,0)</f>
@@ -7011,10 +7017,12 @@
     <row r="8">
       <c r="A8" s="42" t="inlineStr">
         <is>
-          <t>Eval 4</t>
-        </is>
-      </c>
-      <c r="B8" s="49" t="n"/>
+          <t>Primera entrega proyecto</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>10</v>
+      </c>
       <c r="C8" s="49" t="n"/>
       <c r="D8" s="20">
         <f>IFERROR(B8*C8/100,0)</f>
@@ -7024,10 +7032,12 @@
     <row r="9">
       <c r="A9" s="42" t="inlineStr">
         <is>
-          <t>Eval 5</t>
-        </is>
-      </c>
-      <c r="B9" s="49" t="n"/>
+          <t>Entrega final proyecto</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>30</v>
+      </c>
       <c r="C9" s="49" t="n"/>
       <c r="D9" s="20">
         <f>IFERROR(B9*C9/100,0)</f>
@@ -7144,7 +7154,7 @@
     <row r="19">
       <c r="A19" s="47" t="inlineStr">
         <is>
-          <t>MATERIA: Materia obligatoria 1</t>
+          <t>MATERIA: Uitoto</t>
         </is>
       </c>
     </row>
@@ -7173,10 +7183,12 @@
     <row r="21">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>Eval 1</t>
-        </is>
-      </c>
-      <c r="B21" s="49" t="n"/>
+          <t>Mito</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>30</v>
+      </c>
       <c r="C21" s="49" t="n"/>
       <c r="D21" s="20">
         <f>IFERROR(B21*C21/100,0)</f>
@@ -7186,10 +7198,12 @@
     <row r="22">
       <c r="A22" s="42" t="inlineStr">
         <is>
-          <t>Eval 2</t>
-        </is>
-      </c>
-      <c r="B22" s="49" t="n"/>
+          <t>Talleres grupales</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>30</v>
+      </c>
       <c r="C22" s="49" t="n"/>
       <c r="D22" s="20">
         <f>IFERROR(B22*C22/100,0)</f>
@@ -7199,10 +7213,12 @@
     <row r="23">
       <c r="A23" s="42" t="inlineStr">
         <is>
-          <t>Eval 3</t>
-        </is>
-      </c>
-      <c r="B23" s="49" t="n"/>
+          <t>Propuesta final</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>40</v>
+      </c>
       <c r="C23" s="49" t="n"/>
       <c r="D23" s="20">
         <f>IFERROR(B23*C23/100,0)</f>
@@ -7345,7 +7361,7 @@
     <row r="35">
       <c r="A35" s="47" t="inlineStr">
         <is>
-          <t>MATERIA: Materia obligatoria 2</t>
+          <t>MATERIA: PEPI</t>
         </is>
       </c>
     </row>
@@ -7374,10 +7390,12 @@
     <row r="37">
       <c r="A37" s="42" t="inlineStr">
         <is>
-          <t>Eval 1</t>
-        </is>
-      </c>
-      <c r="B37" s="49" t="n"/>
+          <t>Parcial 1</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C37" s="49" t="n"/>
       <c r="D37" s="20">
         <f>IFERROR(B37*C37/100,0)</f>
@@ -7387,10 +7405,12 @@
     <row r="38">
       <c r="A38" s="42" t="inlineStr">
         <is>
-          <t>Eval 2</t>
-        </is>
-      </c>
-      <c r="B38" s="49" t="n"/>
+          <t>Talleres</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="n">
+        <v>40</v>
+      </c>
       <c r="C38" s="49" t="n"/>
       <c r="D38" s="20">
         <f>IFERROR(B38*C38/100,0)</f>
@@ -7400,10 +7420,12 @@
     <row r="39">
       <c r="A39" s="42" t="inlineStr">
         <is>
-          <t>Eval 3</t>
-        </is>
-      </c>
-      <c r="B39" s="49" t="n"/>
+          <t>Quices</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>10</v>
+      </c>
       <c r="C39" s="49" t="n"/>
       <c r="D39" s="20">
         <f>IFERROR(B39*C39/100,0)</f>
@@ -7413,10 +7435,12 @@
     <row r="40">
       <c r="A40" s="42" t="inlineStr">
         <is>
-          <t>Eval 4</t>
-        </is>
-      </c>
-      <c r="B40" s="49" t="n"/>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
+        <v>30</v>
+      </c>
       <c r="C40" s="49" t="n"/>
       <c r="D40" s="20">
         <f>IFERROR(B40*C40/100,0)</f>
@@ -7546,7 +7570,7 @@
     <row r="51">
       <c r="A51" s="47" t="inlineStr">
         <is>
-          <t>MATERIA: Materia obligatoria 3</t>
+          <t>MATERIA: Saneamiento Ambiental</t>
         </is>
       </c>
     </row>
@@ -7575,10 +7599,12 @@
     <row r="53">
       <c r="A53" s="42" t="inlineStr">
         <is>
-          <t>Eval 1</t>
-        </is>
-      </c>
-      <c r="B53" s="49" t="n"/>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B53" s="20" t="n">
+        <v>40</v>
+      </c>
       <c r="C53" s="49" t="n"/>
       <c r="D53" s="20">
         <f>IFERROR(B53*C53/100,0)</f>
@@ -7588,10 +7614,12 @@
     <row r="54">
       <c r="A54" s="42" t="inlineStr">
         <is>
-          <t>Eval 2</t>
-        </is>
-      </c>
-      <c r="B54" s="49" t="n"/>
+          <t>Talleres</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="n">
+        <v>35</v>
+      </c>
       <c r="C54" s="49" t="n"/>
       <c r="D54" s="20">
         <f>IFERROR(B54*C54/100,0)</f>
@@ -7601,10 +7629,12 @@
     <row r="55">
       <c r="A55" s="42" t="inlineStr">
         <is>
-          <t>Eval 3</t>
-        </is>
-      </c>
-      <c r="B55" s="49" t="n"/>
+          <t>Quices</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>15</v>
+      </c>
       <c r="C55" s="49" t="n"/>
       <c r="D55" s="20">
         <f>IFERROR(B55*C55/100,0)</f>
@@ -7614,10 +7644,12 @@
     <row r="56">
       <c r="A56" s="42" t="inlineStr">
         <is>
-          <t>Eval 4</t>
-        </is>
-      </c>
-      <c r="B56" s="49" t="n"/>
+          <t>Participacion</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="n">
+        <v>10</v>
+      </c>
       <c r="C56" s="49" t="n"/>
       <c r="D56" s="20">
         <f>IFERROR(B56*C56/100,0)</f>
@@ -7747,7 +7779,7 @@
     <row r="67">
       <c r="A67" s="47" t="inlineStr">
         <is>
-          <t>MATERIA: Materia optativa 1</t>
+          <t>MATERIA: Alcantarillados</t>
         </is>
       </c>
     </row>
@@ -7776,10 +7808,12 @@
     <row r="69">
       <c r="A69" s="42" t="inlineStr">
         <is>
-          <t>Eval 1</t>
-        </is>
-      </c>
-      <c r="B69" s="49" t="n"/>
+          <t>Informe de salida</t>
+        </is>
+      </c>
+      <c r="B69" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C69" s="49" t="n"/>
       <c r="D69" s="20">
         <f>IFERROR(B69*C69/100,0)</f>
@@ -7789,10 +7823,12 @@
     <row r="70">
       <c r="A70" s="42" t="inlineStr">
         <is>
-          <t>Eval 2</t>
-        </is>
-      </c>
-      <c r="B70" s="49" t="n"/>
+          <t>Planes de gobierno</t>
+        </is>
+      </c>
+      <c r="B70" s="20" t="n">
+        <v>10</v>
+      </c>
       <c r="C70" s="49" t="n"/>
       <c r="D70" s="20">
         <f>IFERROR(B70*C70/100,0)</f>
@@ -7802,10 +7838,12 @@
     <row r="71">
       <c r="A71" s="42" t="inlineStr">
         <is>
-          <t>Eval 3</t>
-        </is>
-      </c>
-      <c r="B71" s="49" t="n"/>
+          <t>Parcial 1</t>
+        </is>
+      </c>
+      <c r="B71" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C71" s="49" t="n"/>
       <c r="D71" s="20">
         <f>IFERROR(B71*C71/100,0)</f>
@@ -7815,10 +7853,12 @@
     <row r="72">
       <c r="A72" s="42" t="inlineStr">
         <is>
-          <t>Eval 4</t>
-        </is>
-      </c>
-      <c r="B72" s="49" t="n"/>
+          <t>Parcial 2</t>
+        </is>
+      </c>
+      <c r="B72" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C72" s="49" t="n"/>
       <c r="D72" s="20">
         <f>IFERROR(B72*C72/100,0)</f>
@@ -7828,10 +7868,12 @@
     <row r="73">
       <c r="A73" s="42" t="inlineStr">
         <is>
-          <t>Eval 5</t>
-        </is>
-      </c>
-      <c r="B73" s="49" t="n"/>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B73" s="20" t="n">
+        <v>30</v>
+      </c>
       <c r="C73" s="49" t="n"/>
       <c r="D73" s="20">
         <f>IFERROR(B73*C73/100,0)</f>
@@ -7948,7 +7990,7 @@
     <row r="83">
       <c r="A83" s="47" t="inlineStr">
         <is>
-          <t>MATERIA: Materia optativa 2</t>
+          <t>MATERIA: Fundamentos de Construccion</t>
         </is>
       </c>
     </row>
@@ -7977,10 +8019,12 @@
     <row r="85">
       <c r="A85" s="42" t="inlineStr">
         <is>
-          <t>Eval 1</t>
-        </is>
-      </c>
-      <c r="B85" s="49" t="n"/>
+          <t>Parcial 1</t>
+        </is>
+      </c>
+      <c r="B85" s="20" t="n">
+        <v>25</v>
+      </c>
       <c r="C85" s="49" t="n"/>
       <c r="D85" s="20">
         <f>IFERROR(B85*C85/100,0)</f>
@@ -7990,10 +8034,12 @@
     <row r="86">
       <c r="A86" s="42" t="inlineStr">
         <is>
-          <t>Eval 2</t>
-        </is>
-      </c>
-      <c r="B86" s="49" t="n"/>
+          <t>Parcial 2</t>
+        </is>
+      </c>
+      <c r="B86" s="20" t="n">
+        <v>25</v>
+      </c>
       <c r="C86" s="49" t="n"/>
       <c r="D86" s="20">
         <f>IFERROR(B86*C86/100,0)</f>
@@ -8003,10 +8049,12 @@
     <row r="87">
       <c r="A87" s="42" t="inlineStr">
         <is>
-          <t>Eval 3</t>
-        </is>
-      </c>
-      <c r="B87" s="49" t="n"/>
+          <t>Proyecto 1</t>
+        </is>
+      </c>
+      <c r="B87" s="20" t="n">
+        <v>20</v>
+      </c>
       <c r="C87" s="49" t="n"/>
       <c r="D87" s="20">
         <f>IFERROR(B87*C87/100,0)</f>
@@ -8016,10 +8064,12 @@
     <row r="88">
       <c r="A88" s="42" t="inlineStr">
         <is>
-          <t>Eval 4</t>
-        </is>
-      </c>
-      <c r="B88" s="49" t="n"/>
+          <t>Talleres</t>
+        </is>
+      </c>
+      <c r="B88" s="20" t="n">
+        <v>30</v>
+      </c>
       <c r="C88" s="49" t="n"/>
       <c r="D88" s="20">
         <f>IFERROR(B88*C88/100,0)</f>
@@ -8236,16 +8286,16 @@
       </c>
       <c r="B3" s="42" t="inlineStr">
         <is>
-          <t>Entrega parcial del proyecto</t>
+          <t>Parcial 1</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>Proyecto</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="D3" s="56" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E3" s="57" t="n"/>
       <c r="F3" s="20">
@@ -8270,16 +8320,16 @@
       </c>
       <c r="B4" s="42" t="inlineStr">
         <is>
-          <t>Sustentacion final</t>
+          <t>Parcial 2</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>Proyecto</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="D4" s="56" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E4" s="57" t="n"/>
       <c r="F4" s="20">
@@ -8297,48 +8347,102 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="42" t="n"/>
-      <c r="B5" s="42" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="56" t="n"/>
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>Diseno Estructural</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="inlineStr">
+        <is>
+          <t>Parcial 3</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D5" s="56" t="n">
+        <v>20</v>
+      </c>
       <c r="E5" s="57" t="n"/>
       <c r="F5" s="20">
         <f>IF(E5="","",E5-TODAY())</f>
         <v/>
       </c>
-      <c r="G5" s="20" t="n"/>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H5" s="20">
         <f>IF(G5="Entregado","Listo",IF(E5="","",IF(F5&lt;0,"VENCIDO",IF(F5&lt;=3,"Vence pronto",IF(F5&lt;=7,"Esta semana","Mas adelante")))))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="42" t="n"/>
-      <c r="B6" s="42" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="56" t="n"/>
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>Diseno Estructural</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>Primera entrega proyecto</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D6" s="56" t="n">
+        <v>10</v>
+      </c>
       <c r="E6" s="57" t="n"/>
       <c r="F6" s="20">
         <f>IF(E6="","",E6-TODAY())</f>
         <v/>
       </c>
-      <c r="G6" s="20" t="n"/>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H6" s="20">
         <f>IF(G6="Entregado","Listo",IF(E6="","",IF(F6&lt;0,"VENCIDO",IF(F6&lt;=3,"Vence pronto",IF(F6&lt;=7,"Esta semana","Mas adelante")))))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="42" t="n"/>
-      <c r="B7" s="42" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="56" t="n"/>
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>Diseno Estructural</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="inlineStr">
+        <is>
+          <t>Entrega final proyecto</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D7" s="56" t="n">
+        <v>30</v>
+      </c>
       <c r="E7" s="57" t="n"/>
       <c r="F7" s="20">
         <f>IF(E7="","",E7-TODAY())</f>
         <v/>
       </c>
-      <c r="G7" s="20" t="n"/>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H7" s="20">
         <f>IF(G7="Entregado","Listo",IF(E7="","",IF(F7&lt;0,"VENCIDO",IF(F7&lt;=3,"Vence pronto",IF(F7&lt;=7,"Esta semana","Mas adelante")))))</f>
         <v/>

</xml_diff>

<commit_message>
Creditos 3 por materia + calculadora de PAPA proyectado con tabla de sensibilidad
Co-authored-by: saospinap-bit <294225962+saospinap-bit@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mi-Sistema-de-Vida.xlsx
+++ b/Mi-Sistema-de-Vida.xlsx
@@ -37,9 +37,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -379,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -403,7 +405,7 @@
     <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -539,30 +541,45 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="13" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="15" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -586,7 +603,7 @@
     <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="19" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1217,7 +1234,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="65" t="inlineStr">
+      <c r="A1" s="70" t="inlineStr">
         <is>
           <t>EGRESOS DEL MES</t>
         </is>
@@ -1262,7 +1279,7 @@
           <t>Transporte</t>
         </is>
       </c>
-      <c r="D3" s="63" t="n">
+      <c r="D3" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -1283,7 +1300,7 @@
           <t>Comida</t>
         </is>
       </c>
-      <c r="D4" s="63" t="n">
+      <c r="D4" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -1304,7 +1321,7 @@
           <t>Salud</t>
         </is>
       </c>
-      <c r="D5" s="63" t="n">
+      <c r="D5" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1325,7 +1342,7 @@
           <t>Educacion</t>
         </is>
       </c>
-      <c r="D6" s="63" t="n">
+      <c r="D6" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -1346,7 +1363,7 @@
           <t>Educacion</t>
         </is>
       </c>
-      <c r="D7" s="63" t="n">
+      <c r="D7" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1367,7 +1384,7 @@
           <t>Ocio</t>
         </is>
       </c>
-      <c r="D8" s="63" t="n">
+      <c r="D8" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="20" t="inlineStr">
@@ -1388,7 +1405,7 @@
           <t>Ocio</t>
         </is>
       </c>
-      <c r="D9" s="63" t="n">
+      <c r="D9" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1401,126 +1418,126 @@
       <c r="A10" s="20" t="n"/>
       <c r="B10" s="42" t="n"/>
       <c r="C10" s="20" t="n"/>
-      <c r="D10" s="63" t="n"/>
+      <c r="D10" s="68" t="n"/>
       <c r="E10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n"/>
       <c r="B11" s="42" t="n"/>
       <c r="C11" s="20" t="n"/>
-      <c r="D11" s="63" t="n"/>
+      <c r="D11" s="68" t="n"/>
       <c r="E11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n"/>
       <c r="B12" s="42" t="n"/>
       <c r="C12" s="20" t="n"/>
-      <c r="D12" s="63" t="n"/>
+      <c r="D12" s="68" t="n"/>
       <c r="E12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n"/>
       <c r="B13" s="42" t="n"/>
       <c r="C13" s="20" t="n"/>
-      <c r="D13" s="63" t="n"/>
+      <c r="D13" s="68" t="n"/>
       <c r="E13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n"/>
       <c r="B14" s="42" t="n"/>
       <c r="C14" s="20" t="n"/>
-      <c r="D14" s="63" t="n"/>
+      <c r="D14" s="68" t="n"/>
       <c r="E14" s="20" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n"/>
       <c r="B15" s="42" t="n"/>
       <c r="C15" s="20" t="n"/>
-      <c r="D15" s="63" t="n"/>
+      <c r="D15" s="68" t="n"/>
       <c r="E15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n"/>
       <c r="B16" s="42" t="n"/>
       <c r="C16" s="20" t="n"/>
-      <c r="D16" s="63" t="n"/>
+      <c r="D16" s="68" t="n"/>
       <c r="E16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n"/>
       <c r="B17" s="42" t="n"/>
       <c r="C17" s="20" t="n"/>
-      <c r="D17" s="63" t="n"/>
+      <c r="D17" s="68" t="n"/>
       <c r="E17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n"/>
       <c r="B18" s="42" t="n"/>
       <c r="C18" s="20" t="n"/>
-      <c r="D18" s="63" t="n"/>
+      <c r="D18" s="68" t="n"/>
       <c r="E18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n"/>
       <c r="B19" s="42" t="n"/>
       <c r="C19" s="20" t="n"/>
-      <c r="D19" s="63" t="n"/>
+      <c r="D19" s="68" t="n"/>
       <c r="E19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n"/>
       <c r="B20" s="42" t="n"/>
       <c r="C20" s="20" t="n"/>
-      <c r="D20" s="63" t="n"/>
+      <c r="D20" s="68" t="n"/>
       <c r="E20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n"/>
       <c r="B21" s="42" t="n"/>
       <c r="C21" s="20" t="n"/>
-      <c r="D21" s="63" t="n"/>
+      <c r="D21" s="68" t="n"/>
       <c r="E21" s="20" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n"/>
       <c r="B22" s="42" t="n"/>
       <c r="C22" s="20" t="n"/>
-      <c r="D22" s="63" t="n"/>
+      <c r="D22" s="68" t="n"/>
       <c r="E22" s="20" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
       <c r="B23" s="42" t="n"/>
       <c r="C23" s="20" t="n"/>
-      <c r="D23" s="63" t="n"/>
+      <c r="D23" s="68" t="n"/>
       <c r="E23" s="20" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="20" t="n"/>
       <c r="B24" s="42" t="n"/>
       <c r="C24" s="20" t="n"/>
-      <c r="D24" s="63" t="n"/>
+      <c r="D24" s="68" t="n"/>
       <c r="E24" s="20" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="20" t="n"/>
       <c r="B25" s="42" t="n"/>
       <c r="C25" s="20" t="n"/>
-      <c r="D25" s="63" t="n"/>
+      <c r="D25" s="68" t="n"/>
       <c r="E25" s="20" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="20" t="n"/>
       <c r="B26" s="42" t="n"/>
       <c r="C26" s="20" t="n"/>
-      <c r="D26" s="63" t="n"/>
+      <c r="D26" s="68" t="n"/>
       <c r="E26" s="20" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="20" t="n"/>
       <c r="B27" s="42" t="n"/>
       <c r="C27" s="20" t="n"/>
-      <c r="D27" s="63" t="n"/>
+      <c r="D27" s="68" t="n"/>
       <c r="E27" s="20" t="n"/>
     </row>
     <row r="28">
@@ -1529,18 +1546,18 @@
           <t>TOTAL EGRESOS</t>
         </is>
       </c>
-      <c r="D28" s="66">
+      <c r="D28" s="71">
         <f>SUM(D3:D27)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="C29" s="67" t="inlineStr">
+      <c r="C29" s="72" t="inlineStr">
         <is>
           <t>Gasto evitable (No)</t>
         </is>
       </c>
-      <c r="D29" s="68">
+      <c r="D29" s="73">
         <f>SUMIF(E3:E27,"No",D3:D27)</f>
         <v/>
       </c>
@@ -1572,7 +1589,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>DEUDAS Y PLAN DE PAGO</t>
         </is>
@@ -1617,10 +1634,10 @@
     </row>
     <row r="3">
       <c r="A3" s="42" t="n"/>
-      <c r="B3" s="63" t="n"/>
-      <c r="C3" s="63" t="n"/>
+      <c r="B3" s="68" t="n"/>
+      <c r="C3" s="68" t="n"/>
       <c r="D3" s="20" t="n"/>
-      <c r="E3" s="63" t="n"/>
+      <c r="E3" s="68" t="n"/>
       <c r="F3" s="20">
         <f>IFERROR(IF(E3=0,"-",ROUNDUP(C3/E3,0)),"-")</f>
         <v/>
@@ -1632,10 +1649,10 @@
     </row>
     <row r="4">
       <c r="A4" s="42" t="n"/>
-      <c r="B4" s="63" t="n"/>
-      <c r="C4" s="63" t="n"/>
+      <c r="B4" s="68" t="n"/>
+      <c r="C4" s="68" t="n"/>
       <c r="D4" s="20" t="n"/>
-      <c r="E4" s="63" t="n"/>
+      <c r="E4" s="68" t="n"/>
       <c r="F4" s="20">
         <f>IFERROR(IF(E4=0,"-",ROUNDUP(C4/E4,0)),"-")</f>
         <v/>
@@ -1647,10 +1664,10 @@
     </row>
     <row r="5">
       <c r="A5" s="42" t="n"/>
-      <c r="B5" s="63" t="n"/>
-      <c r="C5" s="63" t="n"/>
+      <c r="B5" s="68" t="n"/>
+      <c r="C5" s="68" t="n"/>
       <c r="D5" s="20" t="n"/>
-      <c r="E5" s="63" t="n"/>
+      <c r="E5" s="68" t="n"/>
       <c r="F5" s="20">
         <f>IFERROR(IF(E5=0,"-",ROUNDUP(C5/E5,0)),"-")</f>
         <v/>
@@ -1662,10 +1679,10 @@
     </row>
     <row r="6">
       <c r="A6" s="42" t="n"/>
-      <c r="B6" s="63" t="n"/>
-      <c r="C6" s="63" t="n"/>
+      <c r="B6" s="68" t="n"/>
+      <c r="C6" s="68" t="n"/>
       <c r="D6" s="20" t="n"/>
-      <c r="E6" s="63" t="n"/>
+      <c r="E6" s="68" t="n"/>
       <c r="F6" s="20">
         <f>IFERROR(IF(E6=0,"-",ROUNDUP(C6/E6,0)),"-")</f>
         <v/>
@@ -1677,10 +1694,10 @@
     </row>
     <row r="7">
       <c r="A7" s="42" t="n"/>
-      <c r="B7" s="63" t="n"/>
-      <c r="C7" s="63" t="n"/>
+      <c r="B7" s="68" t="n"/>
+      <c r="C7" s="68" t="n"/>
       <c r="D7" s="20" t="n"/>
-      <c r="E7" s="63" t="n"/>
+      <c r="E7" s="68" t="n"/>
       <c r="F7" s="20">
         <f>IFERROR(IF(E7=0,"-",ROUNDUP(C7/E7,0)),"-")</f>
         <v/>
@@ -1692,10 +1709,10 @@
     </row>
     <row r="8">
       <c r="A8" s="42" t="n"/>
-      <c r="B8" s="63" t="n"/>
-      <c r="C8" s="63" t="n"/>
+      <c r="B8" s="68" t="n"/>
+      <c r="C8" s="68" t="n"/>
       <c r="D8" s="20" t="n"/>
-      <c r="E8" s="63" t="n"/>
+      <c r="E8" s="68" t="n"/>
       <c r="F8" s="20">
         <f>IFERROR(IF(E8=0,"-",ROUNDUP(C8/E8,0)),"-")</f>
         <v/>
@@ -1707,10 +1724,10 @@
     </row>
     <row r="9">
       <c r="A9" s="42" t="n"/>
-      <c r="B9" s="63" t="n"/>
-      <c r="C9" s="63" t="n"/>
+      <c r="B9" s="68" t="n"/>
+      <c r="C9" s="68" t="n"/>
       <c r="D9" s="20" t="n"/>
-      <c r="E9" s="63" t="n"/>
+      <c r="E9" s="68" t="n"/>
       <c r="F9" s="20">
         <f>IFERROR(IF(E9=0,"-",ROUNDUP(C9/E9,0)),"-")</f>
         <v/>
@@ -1722,10 +1739,10 @@
     </row>
     <row r="10">
       <c r="A10" s="42" t="n"/>
-      <c r="B10" s="63" t="n"/>
-      <c r="C10" s="63" t="n"/>
+      <c r="B10" s="68" t="n"/>
+      <c r="C10" s="68" t="n"/>
       <c r="D10" s="20" t="n"/>
-      <c r="E10" s="63" t="n"/>
+      <c r="E10" s="68" t="n"/>
       <c r="F10" s="20">
         <f>IFERROR(IF(E10=0,"-",ROUNDUP(C10/E10,0)),"-")</f>
         <v/>
@@ -1737,10 +1754,10 @@
     </row>
     <row r="11">
       <c r="A11" s="42" t="n"/>
-      <c r="B11" s="63" t="n"/>
-      <c r="C11" s="63" t="n"/>
+      <c r="B11" s="68" t="n"/>
+      <c r="C11" s="68" t="n"/>
       <c r="D11" s="20" t="n"/>
-      <c r="E11" s="63" t="n"/>
+      <c r="E11" s="68" t="n"/>
       <c r="F11" s="20">
         <f>IFERROR(IF(E11=0,"-",ROUNDUP(C11/E11,0)),"-")</f>
         <v/>
@@ -1752,10 +1769,10 @@
     </row>
     <row r="12">
       <c r="A12" s="42" t="n"/>
-      <c r="B12" s="63" t="n"/>
-      <c r="C12" s="63" t="n"/>
+      <c r="B12" s="68" t="n"/>
+      <c r="C12" s="68" t="n"/>
       <c r="D12" s="20" t="n"/>
-      <c r="E12" s="63" t="n"/>
+      <c r="E12" s="68" t="n"/>
       <c r="F12" s="20">
         <f>IFERROR(IF(E12=0,"-",ROUNDUP(C12/E12,0)),"-")</f>
         <v/>
@@ -1767,10 +1784,10 @@
     </row>
     <row r="13">
       <c r="A13" s="42" t="n"/>
-      <c r="B13" s="63" t="n"/>
-      <c r="C13" s="63" t="n"/>
+      <c r="B13" s="68" t="n"/>
+      <c r="C13" s="68" t="n"/>
       <c r="D13" s="20" t="n"/>
-      <c r="E13" s="63" t="n"/>
+      <c r="E13" s="68" t="n"/>
       <c r="F13" s="20">
         <f>IFERROR(IF(E13=0,"-",ROUNDUP(C13/E13,0)),"-")</f>
         <v/>
@@ -1782,10 +1799,10 @@
     </row>
     <row r="14">
       <c r="A14" s="42" t="n"/>
-      <c r="B14" s="63" t="n"/>
-      <c r="C14" s="63" t="n"/>
+      <c r="B14" s="68" t="n"/>
+      <c r="C14" s="68" t="n"/>
       <c r="D14" s="20" t="n"/>
-      <c r="E14" s="63" t="n"/>
+      <c r="E14" s="68" t="n"/>
       <c r="F14" s="20">
         <f>IFERROR(IF(E14=0,"-",ROUNDUP(C14/E14,0)),"-")</f>
         <v/>
@@ -1801,13 +1818,13 @@
           <t>DEUDA TOTAL</t>
         </is>
       </c>
-      <c r="C15" s="70">
+      <c r="C15" s="75">
         <f>SUM(C3:C14)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="61" t="inlineStr">
+      <c r="A17" s="66" t="inlineStr">
         <is>
           <t>Estrategia avalancha: paga primero la deuda de MAYOR tasa. Bola de nieve: la mas pequena primero (motivacion).</t>
         </is>
@@ -1842,7 +1859,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="71" t="inlineStr">
+      <c r="A1" s="76" t="inlineStr">
         <is>
           <t>PRESUPUESTO 50 / 30 / 20</t>
         </is>
@@ -1854,7 +1871,7 @@
           <t>Ingreso mensual total</t>
         </is>
       </c>
-      <c r="B3" s="68">
+      <c r="B3" s="73">
         <f>Ingresos!D23</f>
         <v/>
       </c>
@@ -1887,10 +1904,10 @@
           <t>Necesidades (50%)</t>
         </is>
       </c>
-      <c r="B6" s="72" t="n">
+      <c r="B6" s="77" t="n">
         <v>0.5</v>
       </c>
-      <c r="C6" s="73">
+      <c r="C6" s="78">
         <f>$B$3*B6</f>
         <v/>
       </c>
@@ -1906,10 +1923,10 @@
           <t>Gustos / ocio (30%)</t>
         </is>
       </c>
-      <c r="B7" s="72" t="n">
+      <c r="B7" s="77" t="n">
         <v>0.3</v>
       </c>
-      <c r="C7" s="73">
+      <c r="C7" s="78">
         <f>$B$3*B7</f>
         <v/>
       </c>
@@ -1925,10 +1942,10 @@
           <t>Ahorro + deudas (20%)</t>
         </is>
       </c>
-      <c r="B8" s="72" t="n">
+      <c r="B8" s="77" t="n">
         <v>0.2</v>
       </c>
-      <c r="C8" s="73">
+      <c r="C8" s="78">
         <f>$B$3*B8</f>
         <v/>
       </c>
@@ -1944,7 +1961,7 @@
           <t>Gasto real del mes</t>
         </is>
       </c>
-      <c r="C10" s="68">
+      <c r="C10" s="73">
         <f>Egresos!D28</f>
         <v/>
       </c>
@@ -1955,7 +1972,7 @@
           <t>BALANCE (ingreso - gasto)</t>
         </is>
       </c>
-      <c r="C11" s="74">
+      <c r="C11" s="79">
         <f>Ingresos!D23-Egresos!D28</f>
         <v/>
       </c>
@@ -1992,7 +2009,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="75" t="inlineStr">
+      <c r="A1" s="80" t="inlineStr">
         <is>
           <t>PLAN DE PASANTIA - PASO A PASO</t>
         </is>
@@ -2218,7 +2235,7 @@
           <t>Progreso del plan</t>
         </is>
       </c>
-      <c r="C16" s="76">
+      <c r="C16" s="81">
         <f>ROUND(COUNTIF(C3:C14,"Hecho")/12,2)</f>
         <v/>
       </c>
@@ -2264,7 +2281,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="77" t="inlineStr">
+      <c r="A1" s="82" t="inlineStr">
         <is>
           <t>RASTREADOR DE APLICACIONES</t>
         </is>
@@ -2739,7 +2756,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="78" t="inlineStr">
+      <c r="A1" s="83" t="inlineStr">
         <is>
           <t>BECAS PARA TU MAESTRIA (revisar fechas cada ano)</t>
         </is>
@@ -3002,7 +3019,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="66" t="inlineStr">
         <is>
           <t>Confirma SIEMPRE fechas en la web oficial; cambian cada ano.</t>
         </is>
@@ -3046,7 +3063,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>MEJORES DESTINOS POR COSTO (2026, confirmar)</t>
         </is>
@@ -3323,14 +3340,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="66" t="inlineStr">
         <is>
           <t>Si el costo manda: Alemania/Austria. Si quieres beca full: Chevening (UK), Fulbright (USA) o Erasmus Mundus.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="79" t="inlineStr">
+      <c r="A14" s="84" t="inlineStr">
         <is>
           <t>Fuentes: mastersportal.com, thecollegemonk.com, leapscholar.com (reformulado).</t>
         </is>
@@ -3362,7 +3379,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="80" t="inlineStr">
+      <c r="A1" s="85" t="inlineStr">
         <is>
           <t>CURSOS ONLINE PARA TU HOJA DE VIDA</t>
         </is>
@@ -3426,7 +3443,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F3" s="81" t="n">
+      <c r="F3" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3456,7 +3473,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F4" s="81" t="n">
+      <c r="F4" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3486,7 +3503,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F5" s="81" t="n">
+      <c r="F5" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3516,7 +3533,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F6" s="81" t="n">
+      <c r="F6" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3546,7 +3563,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F7" s="81" t="n">
+      <c r="F7" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3576,7 +3593,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F8" s="81" t="n">
+      <c r="F8" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3606,7 +3623,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F9" s="81" t="n">
+      <c r="F9" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3636,7 +3653,7 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F10" s="81" t="n">
+      <c r="F10" s="86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3666,12 +3683,12 @@
           <t>Por empezar</t>
         </is>
       </c>
-      <c r="F11" s="81" t="n">
+      <c r="F11" s="86" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="66" t="inlineStr">
         <is>
           <t>Tip: pide 'financial aid' en Coursera para certificados gratis.</t>
         </is>
@@ -3729,7 +3746,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="77" t="inlineStr">
+      <c r="A1" s="82" t="inlineStr">
         <is>
           <t>RUTA HACIA LA MAESTRIA (linea de tiempo)</t>
         </is>
@@ -3961,7 +3978,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="80" t="inlineStr">
+      <c r="A1" s="85" t="inlineStr">
         <is>
           <t>BIBLIOTECA RECOMENDADA PARA TI</t>
         </is>
@@ -4020,7 +4037,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E3" s="81" t="n">
+      <c r="E3" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="42" t="inlineStr">
@@ -4050,7 +4067,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E4" s="81" t="n">
+      <c r="E4" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="42" t="inlineStr">
@@ -4080,7 +4097,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E5" s="81" t="n">
+      <c r="E5" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="42" t="inlineStr">
@@ -4110,7 +4127,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E6" s="81" t="n">
+      <c r="E6" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="42" t="inlineStr">
@@ -4140,7 +4157,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E7" s="81" t="n">
+      <c r="E7" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="42" t="inlineStr">
@@ -4170,7 +4187,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E8" s="81" t="n">
+      <c r="E8" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="42" t="inlineStr">
@@ -4200,7 +4217,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E9" s="81" t="n">
+      <c r="E9" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="42" t="inlineStr">
@@ -4230,7 +4247,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E10" s="81" t="n">
+      <c r="E10" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="42" t="inlineStr">
@@ -4260,7 +4277,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E11" s="81" t="n">
+      <c r="E11" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="42" t="inlineStr">
@@ -4290,7 +4307,7 @@
           <t>Por leer</t>
         </is>
       </c>
-      <c r="E12" s="81" t="n">
+      <c r="E12" s="86" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="42" t="inlineStr">
@@ -5064,7 +5081,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="82" t="inlineStr">
+      <c r="A2" s="87" t="inlineStr">
         <is>
           <t>Tonificar = peso moderado, 10-15 reps, baja controlada, descanso 45-60s. El Box (Mar/Jue) cubre tu cardio.</t>
         </is>
@@ -5553,7 +5570,7 @@
       <c r="E26" s="49" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="61" t="inlineStr">
+      <c r="A28" s="66" t="inlineStr">
         <is>
           <t>Progresion: sube un poco el peso cada 2 semanas si completas todas las reps con buena tecnica.</t>
         </is>
@@ -5588,14 +5605,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="77" t="inlineStr">
+      <c r="A1" s="82" t="inlineStr">
         <is>
           <t>PLAN DE COMIDAS DIARIO (enfoque tonificar)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="82" t="inlineStr">
+      <c r="A2" s="87" t="inlineStr">
         <is>
           <t>Proteina en cada comida + carbohidrato bueno + verduras. Ajusta porciones a tu hambre. 2-2.5 L de agua al dia.</t>
         </is>
@@ -5883,7 +5900,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="83" t="inlineStr">
+      <c r="A1" s="88" t="inlineStr">
         <is>
           <t>LISTA DE MERCADO SEMANAL</t>
         </is>
@@ -5932,7 +5949,7 @@
           <t>30 und</t>
         </is>
       </c>
-      <c r="D3" s="63" t="n">
+      <c r="D3" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="20" t="inlineStr"/>
@@ -5953,7 +5970,7 @@
           <t>1.5 kg</t>
         </is>
       </c>
-      <c r="D4" s="63" t="n">
+      <c r="D4" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="20" t="inlineStr"/>
@@ -5974,7 +5991,7 @@
           <t>1 kg</t>
         </is>
       </c>
-      <c r="D5" s="63" t="n">
+      <c r="D5" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="20" t="inlineStr"/>
@@ -5995,7 +6012,7 @@
           <t>4 latas / 0.5 kg</t>
         </is>
       </c>
-      <c r="D6" s="63" t="n">
+      <c r="D6" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="20" t="inlineStr"/>
@@ -6016,7 +6033,7 @@
           <t>500 g</t>
         </is>
       </c>
-      <c r="D7" s="63" t="n">
+      <c r="D7" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="20" t="inlineStr"/>
@@ -6037,7 +6054,7 @@
           <t>1 bolsa</t>
         </is>
       </c>
-      <c r="D8" s="63" t="n">
+      <c r="D8" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="20" t="inlineStr"/>
@@ -6058,7 +6075,7 @@
           <t>1 kg</t>
         </is>
       </c>
-      <c r="D9" s="63" t="n">
+      <c r="D9" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="20" t="inlineStr"/>
@@ -6079,7 +6096,7 @@
           <t>500 g</t>
         </is>
       </c>
-      <c r="D10" s="63" t="n">
+      <c r="D10" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="20" t="inlineStr"/>
@@ -6100,7 +6117,7 @@
           <t>1 paquete</t>
         </is>
       </c>
-      <c r="D11" s="63" t="n">
+      <c r="D11" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="20" t="inlineStr"/>
@@ -6121,7 +6138,7 @@
           <t>1 paquete</t>
         </is>
       </c>
-      <c r="D12" s="63" t="n">
+      <c r="D12" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="20" t="inlineStr"/>
@@ -6142,7 +6159,7 @@
           <t>2 kg</t>
         </is>
       </c>
-      <c r="D13" s="63" t="n">
+      <c r="D13" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="20" t="inlineStr"/>
@@ -6163,7 +6180,7 @@
           <t>250 g</t>
         </is>
       </c>
-      <c r="D14" s="63" t="n">
+      <c r="D14" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="20" t="inlineStr"/>
@@ -6184,7 +6201,7 @@
           <t>1 racimo</t>
         </is>
       </c>
-      <c r="D15" s="63" t="n">
+      <c r="D15" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="20" t="inlineStr"/>
@@ -6205,7 +6222,7 @@
           <t>6 und</t>
         </is>
       </c>
-      <c r="D16" s="63" t="n">
+      <c r="D16" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="20" t="inlineStr"/>
@@ -6226,7 +6243,7 @@
           <t>variado</t>
         </is>
       </c>
-      <c r="D17" s="63" t="n">
+      <c r="D17" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="20" t="inlineStr"/>
@@ -6247,7 +6264,7 @@
           <t>variado</t>
         </is>
       </c>
-      <c r="D18" s="63" t="n">
+      <c r="D18" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="20" t="inlineStr"/>
@@ -6268,7 +6285,7 @@
           <t>1 kg</t>
         </is>
       </c>
-      <c r="D19" s="63" t="n">
+      <c r="D19" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="20" t="inlineStr"/>
@@ -6289,7 +6306,7 @@
           <t>2 und</t>
         </is>
       </c>
-      <c r="D20" s="63" t="n">
+      <c r="D20" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="20" t="inlineStr"/>
@@ -6310,7 +6327,7 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="D21" s="63" t="n">
+      <c r="D21" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="20" t="inlineStr"/>
@@ -6331,7 +6348,7 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="D22" s="63" t="n">
+      <c r="D22" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="20" t="inlineStr"/>
@@ -6352,7 +6369,7 @@
           <t>250 g</t>
         </is>
       </c>
-      <c r="D23" s="63" t="n">
+      <c r="D23" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="20" t="inlineStr"/>
@@ -6373,7 +6390,7 @@
           <t>1 botella</t>
         </is>
       </c>
-      <c r="D24" s="63" t="n">
+      <c r="D24" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="20" t="inlineStr"/>
@@ -6394,7 +6411,7 @@
           <t>1 paquete</t>
         </is>
       </c>
-      <c r="D25" s="63" t="n">
+      <c r="D25" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="20" t="inlineStr"/>
@@ -6415,7 +6432,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D26" s="63" t="n">
+      <c r="D26" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="20" t="inlineStr"/>
@@ -6426,13 +6443,13 @@
           <t>TOTAL ESTIMADO</t>
         </is>
       </c>
-      <c r="D27" s="84">
+      <c r="D27" s="89">
         <f>SUM(D3:D26)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="61" t="inlineStr">
+      <c r="A29" s="66" t="inlineStr">
         <is>
           <t>Tip: llena el precio una vez y reutiliza la lista cada semana. El total alimenta tu pestana de Egresos.</t>
         </is>
@@ -6699,7 +6716,7 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="20">
         <f>'Calculadora Notas'!D14</f>
@@ -8834,183 +8851,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>PROMEDIO ACUMULADO DE CARRERA (PAPA)</t>
+          <t>PAPA - actual y PROYECTADO tras este semestre</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>Semestre</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>Creditos</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Promedio semestre</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>Aporte</t>
-        </is>
+      <c r="A3" s="42" t="inlineStr">
+        <is>
+          <t>PAPA actual (antes de este semestre)</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
-        <is>
-          <t>Sem 1</t>
-        </is>
-      </c>
-      <c r="B4" s="49" t="n"/>
-      <c r="C4" s="49" t="n"/>
-      <c r="D4" s="20">
-        <f>IFERROR(B4*C4,0)</f>
-        <v/>
+      <c r="A4" s="42" t="inlineStr">
+        <is>
+          <t>% de avance actual</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="n">
+        <v>0.8169999999999999</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>Sem 2</t>
-        </is>
-      </c>
-      <c r="B5" s="49" t="n"/>
-      <c r="C5" s="49" t="n"/>
-      <c r="D5" s="20">
-        <f>IFERROR(B5*C5,0)</f>
-        <v/>
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>Creditos totales del plan (editable)</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="n">
+        <v>180</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>Sem 3</t>
-        </is>
-      </c>
-      <c r="B6" s="49" t="n"/>
-      <c r="C6" s="49" t="n"/>
-      <c r="D6" s="20">
-        <f>IFERROR(B6*C6,0)</f>
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>Creditos ya cursados (calculado)</t>
+        </is>
+      </c>
+      <c r="B6" s="56">
+        <f>ROUND(B4*B5,0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Sem 4</t>
-        </is>
-      </c>
-      <c r="B7" s="49" t="n"/>
-      <c r="C7" s="49" t="n"/>
-      <c r="D7" s="20">
-        <f>IFERROR(B7*C7,0)</f>
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>Promedio de ESTE semestre (de tus notas)</t>
+        </is>
+      </c>
+      <c r="B7" s="61">
+        <f>'Resumen Semestre'!C10</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Sem 5</t>
-        </is>
-      </c>
-      <c r="B8" s="49" t="n"/>
-      <c r="C8" s="49" t="n"/>
-      <c r="D8" s="20">
-        <f>IFERROR(B8*C8,0)</f>
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>Creditos de este semestre</t>
+        </is>
+      </c>
+      <c r="B8" s="56">
+        <f>'Resumen Semestre'!B10</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>Sem 6</t>
-        </is>
-      </c>
-      <c r="B9" s="49" t="n"/>
-      <c r="C9" s="49" t="n"/>
-      <c r="D9" s="20">
-        <f>IFERROR(B9*C9,0)</f>
+      <c r="A9" s="63" t="inlineStr">
+        <is>
+          <t>PAPA PROYECTADO al terminar el semestre</t>
+        </is>
+      </c>
+      <c r="B9" s="64">
+        <f>IFERROR(ROUND((B3*B6+B7*B8)/(B6+B8),2),0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Sem 7</t>
-        </is>
-      </c>
-      <c r="B10" s="49" t="n"/>
-      <c r="C10" s="49" t="n"/>
-      <c r="D10" s="20">
-        <f>IFERROR(B10*C10,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
-        <is>
-          <t>Sem 8</t>
-        </is>
-      </c>
-      <c r="B11" s="49" t="n"/>
-      <c r="C11" s="49" t="n"/>
-      <c r="D11" s="20">
-        <f>IFERROR(B11*C11,0)</f>
+      <c r="A10" s="42" t="inlineStr">
+        <is>
+          <t>Nuevo % de avance</t>
+        </is>
+      </c>
+      <c r="B10" s="62">
+        <f>IFERROR(ROUND((B6+B8)/B5,3),0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>Sem 9</t>
-        </is>
-      </c>
-      <c r="B12" s="49" t="n"/>
-      <c r="C12" s="49">
-        <f>'Resumen Semestre'!C10</f>
-        <v/>
-      </c>
-      <c r="D12" s="20">
-        <f>IFERROR(B12*C12,0)</f>
-        <v/>
+      <c r="A12" s="58" t="inlineStr">
+        <is>
+          <t>SI tu promedio del semestre es...</t>
+        </is>
+      </c>
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t>...tu PAPA quedaria</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="44" t="inlineStr">
-        <is>
-          <t>PAPA CARRERA</t>
-        </is>
-      </c>
-      <c r="B13" s="25">
-        <f>SUM(B4:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="45">
-        <f>IFERROR(ROUND(SUMPRODUCT(B4:B12,C4:C12)/SUM(B4:B12),2),0)</f>
+      <c r="A13" s="65" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="61">
+        <f>IFERROR(ROUND((B3*B6+3.0*B8)/(B6+B8),2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="65" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="B14" s="61">
+        <f>IFERROR(ROUND((B3*B6+3.5*B8)/(B6+B8),2),0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="61" t="inlineStr">
-        <is>
-          <t>Llena creditos y promedio de semestres 1-8. El Sem 9 se calcula solo.</t>
+      <c r="A15" s="65" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="61">
+        <f>IFERROR(ROUND((B3*B6+4.0*B8)/(B6+B8),2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="65" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="B16" s="61">
+        <f>IFERROR(ROUND((B3*B6+4.2*B8)/(B6+B8),2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="65" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="B17" s="61">
+        <f>IFERROR(ROUND((B3*B6+4.5*B8)/(B6+B8),2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="65" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="61">
+        <f>IFERROR(ROUND((B3*B6+5.0*B8)/(B6+B8),2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="66" t="inlineStr">
+        <is>
+          <t>Todas tus materias tienen 3 creditos -&gt; el promedio del semestre = promedio simple de las 6 notas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="66" t="inlineStr">
+        <is>
+          <t>Ajusta 'Creditos totales del plan' si conoces el numero exacto de tu pensum (UNAL Ing. Civil ~180).</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9223,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>INGRESOS DEL MES</t>
         </is>
@@ -9252,7 +9268,7 @@
           <t>Familia</t>
         </is>
       </c>
-      <c r="D3" s="63" t="n">
+      <c r="D3" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -9273,7 +9289,7 @@
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="D4" s="63" t="n">
+      <c r="D4" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -9294,7 +9310,7 @@
           <t>Otro</t>
         </is>
       </c>
-      <c r="D5" s="63" t="n">
+      <c r="D5" s="68" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -9307,119 +9323,119 @@
       <c r="A6" s="20" t="n"/>
       <c r="B6" s="42" t="n"/>
       <c r="C6" s="20" t="n"/>
-      <c r="D6" s="63" t="n"/>
+      <c r="D6" s="68" t="n"/>
       <c r="E6" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n"/>
       <c r="B7" s="42" t="n"/>
       <c r="C7" s="20" t="n"/>
-      <c r="D7" s="63" t="n"/>
+      <c r="D7" s="68" t="n"/>
       <c r="E7" s="20" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="20" t="n"/>
       <c r="B8" s="42" t="n"/>
       <c r="C8" s="20" t="n"/>
-      <c r="D8" s="63" t="n"/>
+      <c r="D8" s="68" t="n"/>
       <c r="E8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n"/>
       <c r="B9" s="42" t="n"/>
       <c r="C9" s="20" t="n"/>
-      <c r="D9" s="63" t="n"/>
+      <c r="D9" s="68" t="n"/>
       <c r="E9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n"/>
       <c r="B10" s="42" t="n"/>
       <c r="C10" s="20" t="n"/>
-      <c r="D10" s="63" t="n"/>
+      <c r="D10" s="68" t="n"/>
       <c r="E10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n"/>
       <c r="B11" s="42" t="n"/>
       <c r="C11" s="20" t="n"/>
-      <c r="D11" s="63" t="n"/>
+      <c r="D11" s="68" t="n"/>
       <c r="E11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n"/>
       <c r="B12" s="42" t="n"/>
       <c r="C12" s="20" t="n"/>
-      <c r="D12" s="63" t="n"/>
+      <c r="D12" s="68" t="n"/>
       <c r="E12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n"/>
       <c r="B13" s="42" t="n"/>
       <c r="C13" s="20" t="n"/>
-      <c r="D13" s="63" t="n"/>
+      <c r="D13" s="68" t="n"/>
       <c r="E13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n"/>
       <c r="B14" s="42" t="n"/>
       <c r="C14" s="20" t="n"/>
-      <c r="D14" s="63" t="n"/>
+      <c r="D14" s="68" t="n"/>
       <c r="E14" s="20" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n"/>
       <c r="B15" s="42" t="n"/>
       <c r="C15" s="20" t="n"/>
-      <c r="D15" s="63" t="n"/>
+      <c r="D15" s="68" t="n"/>
       <c r="E15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n"/>
       <c r="B16" s="42" t="n"/>
       <c r="C16" s="20" t="n"/>
-      <c r="D16" s="63" t="n"/>
+      <c r="D16" s="68" t="n"/>
       <c r="E16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n"/>
       <c r="B17" s="42" t="n"/>
       <c r="C17" s="20" t="n"/>
-      <c r="D17" s="63" t="n"/>
+      <c r="D17" s="68" t="n"/>
       <c r="E17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n"/>
       <c r="B18" s="42" t="n"/>
       <c r="C18" s="20" t="n"/>
-      <c r="D18" s="63" t="n"/>
+      <c r="D18" s="68" t="n"/>
       <c r="E18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n"/>
       <c r="B19" s="42" t="n"/>
       <c r="C19" s="20" t="n"/>
-      <c r="D19" s="63" t="n"/>
+      <c r="D19" s="68" t="n"/>
       <c r="E19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n"/>
       <c r="B20" s="42" t="n"/>
       <c r="C20" s="20" t="n"/>
-      <c r="D20" s="63" t="n"/>
+      <c r="D20" s="68" t="n"/>
       <c r="E20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n"/>
       <c r="B21" s="42" t="n"/>
       <c r="C21" s="20" t="n"/>
-      <c r="D21" s="63" t="n"/>
+      <c r="D21" s="68" t="n"/>
       <c r="E21" s="20" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n"/>
       <c r="B22" s="42" t="n"/>
       <c r="C22" s="20" t="n"/>
-      <c r="D22" s="63" t="n"/>
+      <c r="D22" s="68" t="n"/>
       <c r="E22" s="20" t="n"/>
     </row>
     <row r="23">
@@ -9428,7 +9444,7 @@
           <t>TOTAL INGRESOS</t>
         </is>
       </c>
-      <c r="D23" s="64">
+      <c r="D23" s="69">
         <f>SUM(D3:D22)</f>
         <v/>
       </c>

</xml_diff>